<commit_message>
Add Credifin social media links to dashboard
</commit_message>
<xml_diff>
--- a/data/content.xlsx
+++ b/data/content.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -881,6 +881,43 @@
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
     </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Hello</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Reel</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>dhruv post</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Revert "Add Credifin social media links to dashboard"
This reverts commit 854591bb95d52f3c44ca0f340bbcd692ccd0f75d.
</commit_message>
<xml_diff>
--- a/data/content.xlsx
+++ b/data/content.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -881,43 +881,6 @@
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
     </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Hello</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Instagram</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Reel</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>2026-04-20</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>dhruv post</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>